<commit_message>
Update Emerging Compounder Radar
</commit_message>
<xml_diff>
--- a/data/compounder_radar.xlsx
+++ b/data/compounder_radar.xlsx
@@ -423,19 +423,19 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="8" customWidth="1" min="14" max="14"/>
     <col width="45" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
     <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="23" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
   </cols>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>85.7</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="D2" t="n">
         <v>86</v>
@@ -577,16 +577,16 @@
         <v>0.14119</v>
       </c>
       <c r="J2" t="n">
-        <v>0.2438645371039323</v>
+        <v>0.2076560448920286</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.4090205387552895</v>
+        <v>-0.426223758705346</v>
       </c>
       <c r="L2" t="n">
-        <v>0.596215871814282</v>
+        <v>0.4871996003291405</v>
       </c>
       <c r="M2" t="n">
-        <v>244400128000</v>
+        <v>251727839232</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -605,33 +605,33 @@
         <v>1</v>
       </c>
       <c r="R2" t="n">
-        <v>0.25610937585155</v>
+        <v>0.2761509215274789</v>
       </c>
       <c r="S2" t="n">
-        <v>0.4581985075574582</v>
+        <v>0.4891442076825607</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NVIDIA Corporation</t>
+          <t>Veeva Systems Inc.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>VEEV</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>83.59999999999999</v>
+        <v>78</v>
       </c>
       <c r="D3" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -639,32 +639,32 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1.000450949944396</v>
+        <v>0.1402968452680178</v>
       </c>
       <c r="G3" t="n">
-        <v>2.04239508347386</v>
+        <v>0.2194365698361114</v>
       </c>
       <c r="H3" t="n">
-        <v>0.74674004</v>
+        <v>0.74961</v>
       </c>
       <c r="I3" t="n">
-        <v>0.53572</v>
+        <v>0.07583000500000001</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4200732766105226</v>
+        <v>0.1329889481707318</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.2868987671470742</v>
+        <v>-0.4357850609756097</v>
       </c>
       <c r="L3" t="n">
-        <v>1.464186412467847</v>
+        <v>0.3051709663314389</v>
       </c>
       <c r="M3" t="n">
-        <v>5562502742016</v>
+        <v>42484879360</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -679,33 +679,33 @@
         <v>1</v>
       </c>
       <c r="R3" t="n">
-        <v>0.123159403974308</v>
+        <v>0.6242648649930138</v>
       </c>
       <c r="S3" t="n">
-        <v>0.2970472917197908</v>
+        <v>0.4514077307430893</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sandisk Corporation</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>76.09999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="D4" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -713,109 +713,111 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.4928519097558826</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
+        <v>1.000450949944396</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2.04239508347386</v>
+      </c>
       <c r="H4" t="n">
-        <v>0.71474</v>
+        <v>0.74674004</v>
       </c>
       <c r="I4" t="n">
-        <v>0.43910998</v>
+        <v>0.53572</v>
       </c>
       <c r="J4" t="n">
-        <v>0.221314367816092</v>
+        <v>0.4988207430482385</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.961</v>
+        <v>-0.2474689633056942</v>
       </c>
       <c r="L4" t="n">
-        <v>0.2302959082373486</v>
+        <v>2.015690114772307</v>
       </c>
       <c r="M4" t="n">
-        <v>254769070080</v>
+        <v>5271048421376</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q4" t="b">
         <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>0.1158710591376246</v>
+        <v>0.06669722286781954</v>
       </c>
       <c r="S4" t="n">
-        <v>2.299641483719194</v>
+        <v>0.1946541308810243</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Veeva Systems Inc.</t>
+          <t>Expedia Group, Inc.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>VEEV</t>
+          <t>EXPE</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>74.3</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>High Conviction</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.1402968452680178</v>
+        <v>0.08087962506974211</v>
       </c>
       <c r="G5" t="n">
-        <v>0.2194365698361114</v>
+        <v>0.6534957812135467</v>
       </c>
       <c r="H5" t="n">
-        <v>0.74961</v>
+        <v>0.90433</v>
       </c>
       <c r="I5" t="n">
-        <v>0.07583000500000001</v>
+        <v>0.061079998</v>
       </c>
       <c r="J5" t="n">
-        <v>0.06901039659747732</v>
+        <v>0.2129719047110352</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.4618124977280162</v>
+        <v>-0.3400277748103835</v>
       </c>
       <c r="L5" t="n">
-        <v>0.149433800377834</v>
+        <v>0.6263367891925858</v>
       </c>
       <c r="M5" t="n">
-        <v>44539502592</v>
+        <v>33705799680</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P5" t="n">
@@ -825,62 +827,62 @@
         <v>1</v>
       </c>
       <c r="R5" t="n">
-        <v>0.5937083330349822</v>
+        <v>0.251824158196462</v>
       </c>
       <c r="S5" t="n">
-        <v>0.4071818947670449</v>
+        <v>0.2380054660798332</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Amphenol Corporation</t>
+          <t>Microsoft Corporation</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>73.40000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="D6" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>High Conviction</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.2230660589034148</v>
+        <v>0.1612397915820203</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2972340671812952</v>
+        <v>0.2285599828574523</v>
       </c>
       <c r="H6" t="n">
-        <v>0.38952</v>
+        <v>0.67944</v>
       </c>
       <c r="I6" t="n">
-        <v>0.14473</v>
+        <v>0.14088</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1977175646291374</v>
+        <v>0.1559331759578719</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.3332326648949021</v>
+        <v>-0.2954421645178863</v>
       </c>
       <c r="L6" t="n">
-        <v>0.5933318832698928</v>
+        <v>0.5277959434542107</v>
       </c>
       <c r="M6" t="n">
-        <v>204132728832</v>
+        <v>3680323239936</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -889,7 +891,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P6" t="n">
@@ -899,33 +901,33 @@
         <v>1</v>
       </c>
       <c r="R6" t="n">
-        <v>0.1945088969397628</v>
+        <v>0.2721294926115181</v>
       </c>
       <c r="S6" t="n">
-        <v>0.259858263710129</v>
+        <v>0.2383381805824003</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Micron Technology, Inc.</t>
+          <t>Robinhood Markets, Inc.</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>72.5</v>
+        <v>74.2</v>
       </c>
       <c r="D7" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -933,28 +935,26 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.06713489726936261</v>
-      </c>
-      <c r="G7" t="n">
-        <v>-0.006929629272242499</v>
-      </c>
+        <v>0.4878747583673768</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>0.7256899999999999</v>
+        <v>0.9189000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>0.3487</v>
+        <v>0.04528</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4884182413755791</v>
+        <v>0.1483026561250778</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.8736953934231106</v>
+        <v>-0.4357732966154393</v>
       </c>
       <c r="L7" t="n">
-        <v>0.5590257715128519</v>
+        <v>0.3403206604831313</v>
       </c>
       <c r="M7" t="n">
-        <v>1148129771520</v>
+        <v>101209694208</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -963,40 +963,40 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Høj bruttomargin, positivt momentum, analytiker-upside over 20 %</t>
+          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="Q7" t="b">
         <v>1</v>
       </c>
       <c r="R7" t="n">
-        <v>0.1767761689947756</v>
+        <v>0.2205355697448483</v>
       </c>
       <c r="S7" t="n">
-        <v>1.746890376291639</v>
+        <v>0.4788491281272171</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>Blackstone Inc.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>72.5</v>
+        <v>71.7</v>
       </c>
       <c r="D8" t="n">
         <v>72</v>
@@ -1007,32 +1007,32 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.1612397915820203</v>
+        <v>0.2027465724146367</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2285599828574523</v>
+        <v>0.1792330812083591</v>
       </c>
       <c r="H8" t="n">
-        <v>0.67944</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.14088</v>
+        <v>0.1433</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1465182309385631</v>
+        <v>0.1234997276476542</v>
       </c>
       <c r="K8" t="n">
-        <v>-0.3011807084250551</v>
+        <v>-0.2083884522605244</v>
       </c>
       <c r="L8" t="n">
-        <v>0.486479468438538</v>
+        <v>0.5926418969380151</v>
       </c>
       <c r="M8" t="n">
-        <v>3710545297408</v>
+        <v>153607716864</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1047,30 +1047,30 @@
         <v>1</v>
       </c>
       <c r="R8" t="n">
-        <v>0.2015280836479112</v>
+        <v>0.0739651567046733</v>
       </c>
       <c r="S8" t="n">
-        <v>0.2268315631847659</v>
+        <v>0.2830377383397216</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices, Inc.</t>
+          <t>Mastercard Incorporated</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>71.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="D9" t="n">
         <v>72</v>
@@ -1081,32 +1081,32 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.1364359933536843</v>
+        <v>0.1382198495222513</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4666355102918431</v>
+        <v>0.173598959321368</v>
       </c>
       <c r="H9" t="n">
-        <v>0.55724</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>0.05128</v>
+        <v>0.24063</v>
       </c>
       <c r="J9" t="n">
-        <v>0.2853506292271291</v>
+        <v>0.171337866090409</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.6875431873861424</v>
+        <v>-0.1838929004374639</v>
       </c>
       <c r="L9" t="n">
-        <v>0.415029389371098</v>
+        <v>0.9317263781408222</v>
       </c>
       <c r="M9" t="n">
-        <v>779621105664</v>
+        <v>498616074240</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1121,26 +1121,26 @@
         <v>1</v>
       </c>
       <c r="R9" t="n">
-        <v>0.02399331515985126</v>
+        <v>0.1719062955910109</v>
       </c>
       <c r="S9" t="n">
-        <v>1.48178571689113</v>
+        <v>0.1484264229690482</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Interactive Brokers Group, Inc.</t>
+          <t>Amphenol Corporation</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IBKR</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1155,37 +1155,37 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.3459787421885367</v>
+        <v>0.2230660589034148</v>
       </c>
       <c r="G10" t="n">
-        <v>0.3328887406583814</v>
+        <v>0.2972340671812952</v>
       </c>
       <c r="H10" t="n">
-        <v>0.93036</v>
+        <v>0.38952</v>
       </c>
       <c r="I10" t="n">
-        <v>0.022839999</v>
+        <v>0.14473</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1416374433167782</v>
+        <v>0.1828492612011439</v>
       </c>
       <c r="K10" t="n">
-        <v>-0.3635283955949039</v>
+        <v>-0.3008817921830315</v>
       </c>
       <c r="L10" t="n">
-        <v>0.3896186516186515</v>
+        <v>0.6077112871287126</v>
       </c>
       <c r="M10" t="n">
-        <v>157807394816</v>
+        <v>206943928320</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, positivt momentum</t>
         </is>
       </c>
       <c r="P10" t="n">
@@ -1195,30 +1195,30 @@
         <v>1</v>
       </c>
       <c r="R10" t="n">
-        <v>0.09838686751587034</v>
+        <v>0.1025396709569864</v>
       </c>
       <c r="S10" t="n">
-        <v>0.3912707391772128</v>
+        <v>0.2810940606230861</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Expedia Group, Inc.</t>
+          <t>Salesforce, Inc.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>71.2</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="D11" t="n">
         <v>71</v>
@@ -1229,28 +1229,28 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.08087962506974211</v>
+        <v>0.09820006113830493</v>
       </c>
       <c r="G11" t="n">
-        <v>0.6534957812135467</v>
+        <v>2.336504917866317</v>
       </c>
       <c r="H11" t="n">
-        <v>0.90433</v>
+        <v>0.77282</v>
       </c>
       <c r="I11" t="n">
-        <v>0.061079998</v>
+        <v>0.05704</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1401341095155011</v>
+        <v>0.1035569998385273</v>
       </c>
       <c r="K11" t="n">
-        <v>-0.37813716279694</v>
+        <v>-0.4093331180364929</v>
       </c>
       <c r="L11" t="n">
-        <v>0.3705906832298132</v>
+        <v>0.2529895463510846</v>
       </c>
       <c r="M11" t="n">
-        <v>35771379712</v>
+        <v>203873566720</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1269,30 +1269,30 @@
         <v>1</v>
       </c>
       <c r="R11" t="n">
-        <v>0.3040443142797304</v>
+        <v>0.488254765770479</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1982347273512726</v>
+        <v>0.2494004299711519</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Blackstone Inc.</t>
+          <t>Advanced Micro Devices, Inc.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>70.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="D12" t="n">
         <v>70</v>
@@ -1303,32 +1303,32 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.2027465724146367</v>
+        <v>0.1364359933536843</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1792330812083591</v>
+        <v>0.4666355102918431</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>0.55724</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1433</v>
+        <v>0.05128</v>
       </c>
       <c r="J12" t="n">
-        <v>0.05800675725302962</v>
+        <v>0.1916920155774708</v>
       </c>
       <c r="K12" t="n">
-        <v>-0.2528094013955197</v>
+        <v>-0.7096661693759324</v>
       </c>
       <c r="L12" t="n">
-        <v>0.229448576409064</v>
+        <v>0.2701157584361691</v>
       </c>
       <c r="M12" t="n">
-        <v>162739781632</v>
+        <v>842569351168</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1343,105 +1343,107 @@
         <v>1</v>
       </c>
       <c r="R12" t="n">
-        <v>0.1923610114439704</v>
+        <v>0.0566690387634774</v>
       </c>
       <c r="S12" t="n">
-        <v>0.2573665935775524</v>
+        <v>1.610144586552342</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Palo Alto Networks, Inc.</t>
+          <t>DexCom, Inc.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>DXCM</t>
         </is>
       </c>
       <c r="C13" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="D13" t="n">
         <v>70</v>
       </c>
-      <c r="D13" t="n">
-        <v>66</v>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>Watch</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.1878825003317091</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
+        <v>0.1701360960301399</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.365979383233586</v>
+      </c>
       <c r="H13" t="n">
-        <v>0.70488</v>
+        <v>0.62473</v>
       </c>
       <c r="I13" t="n">
-        <v>0.01746</v>
+        <v>0.103310004</v>
       </c>
       <c r="J13" t="n">
-        <v>0.1717577867130768</v>
+        <v>0.1335661808984705</v>
       </c>
       <c r="K13" t="n">
-        <v>-0.5811978635299766</v>
+        <v>-0.348307840539564</v>
       </c>
       <c r="L13" t="n">
-        <v>0.2955237751045485</v>
+        <v>0.3834716459197789</v>
       </c>
       <c r="M13" t="n">
-        <v>271606906880</v>
+        <v>31332263936</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q13" t="b">
         <v>1</v>
       </c>
       <c r="R13" t="n">
-        <v>0.2249954961190344</v>
+        <v>0.1033886880969683</v>
       </c>
       <c r="S13" t="n">
-        <v>1.019145735254052</v>
+        <v>0.2722953732972837</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mastercard Incorporated</t>
+          <t>Palantir Technologies Inc.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>69.7</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="D14" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1449,73 +1451,71 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.1382198495222513</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0.173598959321368</v>
-      </c>
+        <v>0.3291712528765784</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>0.84796</v>
       </c>
       <c r="I14" t="n">
-        <v>0.24063</v>
+        <v>0.17292999</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1583345418760034</v>
+        <v>0.1704217544698918</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.1980110840627752</v>
+        <v>-0.3639299168809423</v>
       </c>
       <c r="L14" t="n">
-        <v>0.7996246403348145</v>
+        <v>0.4682817942819589</v>
       </c>
       <c r="M14" t="n">
-        <v>507393736704</v>
+        <v>401863442432</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P14" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="Q14" t="b">
         <v>1</v>
       </c>
       <c r="R14" t="n">
-        <v>0.1814388483028617</v>
+        <v>0.2757857292607997</v>
       </c>
       <c r="S14" t="n">
-        <v>0.1126430407173609</v>
+        <v>0.08944622623803955</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Salesforce, Inc.</t>
+          <t>Visa Inc.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>V</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>69.40000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="D15" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1523,37 +1523,37 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.09820006113830493</v>
+        <v>0.1092124213025429</v>
       </c>
       <c r="G15" t="n">
-        <v>2.336504917866317</v>
+        <v>0.1337066930484769</v>
       </c>
       <c r="H15" t="n">
-        <v>0.77282</v>
+        <v>0.97725</v>
       </c>
       <c r="I15" t="n">
-        <v>0.05704</v>
+        <v>0.1911</v>
       </c>
       <c r="J15" t="n">
-        <v>0.0447715156424795</v>
+        <v>0.1320330139020112</v>
       </c>
       <c r="K15" t="n">
-        <v>-0.4355591559618872</v>
+        <v>-0.2066675664732083</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1027908954034183</v>
+        <v>0.6388666405433651</v>
       </c>
       <c r="M15" t="n">
-        <v>213346304000</v>
+        <v>691647676416</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P15" t="n">
@@ -1563,33 +1563,33 @@
         <v>1</v>
       </c>
       <c r="R15" t="n">
-        <v>0.3998657393060088</v>
+        <v>0.1632603895031108</v>
       </c>
       <c r="S15" t="n">
-        <v>0.2891448931981548</v>
+        <v>0.2134015991555402</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DexCom, Inc.</t>
+          <t>DoorDash, Inc.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DXCM</t>
+          <t>DASH</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>69.09999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="D16" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1597,70 +1597,68 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.1701360960301399</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0.365979383233586</v>
-      </c>
+        <v>0.2772574009717286</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>0.62473</v>
+        <v>0.52225</v>
       </c>
       <c r="I16" t="n">
-        <v>0.103310004</v>
+        <v>0.029719999</v>
       </c>
       <c r="J16" t="n">
-        <v>0.07076222980659841</v>
+        <v>0.2630342163901958</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.3844141069397042</v>
+        <v>-0.2904184204010892</v>
       </c>
       <c r="L16" t="n">
-        <v>0.1840781296241492</v>
+        <v>0.905707757885764</v>
       </c>
       <c r="M16" t="n">
-        <v>33170012160</v>
+        <v>87504519168</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="Q16" t="b">
         <v>1</v>
       </c>
       <c r="R16" t="n">
-        <v>0.2064232883548802</v>
+        <v>0.3063587666231378</v>
       </c>
       <c r="S16" t="n">
-        <v>0.2907489500059546</v>
+        <v>0.2485316658314818</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Seagate Technology Holdings PLC</t>
+          <t>Workday, Inc.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>69.09999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D17" t="n">
         <v>66</v>
@@ -1671,26 +1669,26 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.1820341908356484</v>
+        <v>0.1539697807235301</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>0.45576</v>
+        <v>0.75795</v>
       </c>
       <c r="I17" t="n">
-        <v>0.29354998</v>
+        <v>0.04513</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3246514694800302</v>
+        <v>0.1237578890683899</v>
       </c>
       <c r="K17" t="n">
-        <v>-0.7796015448379804</v>
+        <v>-0.4057081313947226</v>
       </c>
       <c r="L17" t="n">
-        <v>0.4164325630569402</v>
+        <v>0.3050416777276349</v>
       </c>
       <c r="M17" t="n">
-        <v>192484655104</v>
+        <v>44753698816</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -1709,30 +1707,30 @@
         <v>1</v>
       </c>
       <c r="R17" t="n">
-        <v>0.002850367079626048</v>
+        <v>0.4226614470611312</v>
       </c>
       <c r="S17" t="n">
-        <v>1.413175079577211</v>
+        <v>0.3843745176173947</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Lam Research Corporation</t>
+          <t>Interactive Brokers Group, Inc.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>IBKR</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>68.3</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="D18" t="n">
         <v>68</v>
@@ -1743,28 +1741,28 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.1005582390165327</v>
+        <v>0.3459787421885367</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2014836612049711</v>
+        <v>0.3328887406583814</v>
       </c>
       <c r="H18" t="n">
-        <v>0.50469</v>
+        <v>0.93036</v>
       </c>
       <c r="I18" t="n">
-        <v>0.22840999</v>
+        <v>0.022839999</v>
       </c>
       <c r="J18" t="n">
-        <v>0.2054964082561352</v>
+        <v>0.1572557732297253</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.6604583130180399</v>
+        <v>-0.3548210572397943</v>
       </c>
       <c r="L18" t="n">
-        <v>0.3111421329789852</v>
+        <v>0.4431974090067858</v>
       </c>
       <c r="M18" t="n">
-        <v>384968884224</v>
+        <v>155677638656</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -1783,33 +1781,33 @@
         <v>1</v>
       </c>
       <c r="R18" t="n">
-        <v>0.01512373068940587</v>
+        <v>0.02952514034916542</v>
       </c>
       <c r="S18" t="n">
-        <v>0.5445076813061343</v>
+        <v>0.3679819960781479</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Robinhood Markets, Inc.</t>
+          <t>Fortinet, Inc.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HOOD</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>68</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1817,26 +1815,28 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.4878747583673768</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
+        <v>0.1546194776009138</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.3167495145145989</v>
+      </c>
       <c r="H19" t="n">
-        <v>0.9189000000000001</v>
+        <v>0.80204004</v>
       </c>
       <c r="I19" t="n">
-        <v>0.04528</v>
+        <v>0.14166</v>
       </c>
       <c r="J19" t="n">
-        <v>0.01036409794447635</v>
+        <v>0.04520407509450886</v>
       </c>
       <c r="K19" t="n">
-        <v>-0.4798542297928098</v>
+        <v>-0.5287371051451272</v>
       </c>
       <c r="L19" t="n">
-        <v>0.02159842990016224</v>
+        <v>0.08549442559379541</v>
       </c>
       <c r="M19" t="n">
-        <v>109786939392</v>
+        <v>114510700544</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -1845,43 +1845,43 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q19" t="b">
         <v>1</v>
       </c>
       <c r="R19" t="n">
-        <v>0.4806596192907207</v>
+        <v>0.07589969633894245</v>
       </c>
       <c r="S19" t="n">
-        <v>0.5839928189273125</v>
+        <v>0.8491706694621828</v>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fortinet, Inc.</t>
+          <t>CrowdStrike Holdings, Inc.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>67.90000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="D20" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1889,28 +1889,26 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.1546194776009138</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0.3167495145145989</v>
-      </c>
+        <v>0.2900686653697968</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>0.80204004</v>
+        <v>0.75185996</v>
       </c>
       <c r="I20" t="n">
-        <v>0.14166</v>
+        <v>-0.0078100003</v>
       </c>
       <c r="J20" t="n">
-        <v>0.0384008573805108</v>
+        <v>0.1322917674373609</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.5294004734787894</v>
+        <v>-0.5855664119183515</v>
       </c>
       <c r="L20" t="n">
-        <v>0.07253649987913988</v>
+        <v>0.2259210308937717</v>
       </c>
       <c r="M20" t="n">
-        <v>114672107520</v>
+        <v>211688292352</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -1919,24 +1917,24 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P20" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="Q20" t="b">
         <v>1</v>
       </c>
       <c r="R20" t="n">
-        <v>0.08024606855191685</v>
+        <v>0.1958410870652747</v>
       </c>
       <c r="S20" t="n">
-        <v>0.8679335091002895</v>
+        <v>0.8728994110813904</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
@@ -1952,10 +1950,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>67.8</v>
+        <v>66</v>
       </c>
       <c r="D21" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1975,20 +1973,20 @@
         <v>0.16832</v>
       </c>
       <c r="J21" t="n">
-        <v>0.002958579881656709</v>
+        <v>0.05161052111632514</v>
       </c>
       <c r="K21" t="n">
-        <v>-0.3602366863905325</v>
+        <v>-0.332427759940726</v>
       </c>
       <c r="L21" t="n">
-        <v>0.008212877792378184</v>
+        <v>0.1552533432392277</v>
       </c>
       <c r="M21" t="n">
-        <v>25691938816</v>
+        <v>24621694976</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -2003,33 +2001,33 @@
         <v>1</v>
       </c>
       <c r="R21" t="n">
-        <v>0.2380348056296557</v>
+        <v>0.1264954016324626</v>
       </c>
       <c r="S21" t="n">
-        <v>0.3211381777628204</v>
+        <v>0.3198957169608165</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Visa Inc.</t>
+          <t>News Corporation</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>NWSA</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>67.5</v>
+        <v>65.5</v>
       </c>
       <c r="D22" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2037,28 +2035,28 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.1092124213025429</v>
+        <v>0.0405993172034298</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1337066930484769</v>
+        <v>0.5822968332827563</v>
       </c>
       <c r="H22" t="n">
-        <v>0.97725</v>
+        <v>0.57167</v>
       </c>
       <c r="I22" t="n">
-        <v>0.1911</v>
+        <v>0.04658</v>
       </c>
       <c r="J22" t="n">
-        <v>0.1180889700589223</v>
+        <v>0.2283457880434783</v>
       </c>
       <c r="K22" t="n">
-        <v>-0.2164395979417175</v>
+        <v>-0.2459239130434783</v>
       </c>
       <c r="L22" t="n">
-        <v>0.5455978073417096</v>
+        <v>0.9285220994475138</v>
       </c>
       <c r="M22" t="n">
-        <v>700273459200</v>
+        <v>15790737408</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -2067,7 +2065,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
+          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P22" t="n">
@@ -2077,33 +2075,33 @@
         <v>1</v>
       </c>
       <c r="R22" t="n">
-        <v>0.1613153107304006</v>
+        <v>0.1231581453609647</v>
       </c>
       <c r="S22" t="n">
-        <v>0.1864941770015818</v>
+        <v>0.2527166676960533</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CrowdStrike Holdings, Inc.</t>
+          <t>ServiceNow, Inc.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>66.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="D23" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2111,26 +2109,28 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.2900686653697968</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
+        <v>0.2237651786474262</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.7345580184539504</v>
+      </c>
       <c r="H23" t="n">
-        <v>0.75185996</v>
+        <v>0.74768996</v>
       </c>
       <c r="I23" t="n">
-        <v>-0.0078100003</v>
+        <v>0.04249</v>
       </c>
       <c r="J23" t="n">
-        <v>0.08653214453308311</v>
+        <v>0.08534233758394327</v>
       </c>
       <c r="K23" t="n">
-        <v>-0.5979352416705772</v>
+        <v>-0.3870067154606505</v>
       </c>
       <c r="L23" t="n">
-        <v>0.1447182545911161</v>
+        <v>0.2205190095535192</v>
       </c>
       <c r="M23" t="n">
-        <v>218200522752</v>
+        <v>137017729024</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -2139,43 +2139,43 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, høj bruttomargin</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q23" t="b">
         <v>1</v>
       </c>
       <c r="R23" t="n">
-        <v>0.2703049083535807</v>
+        <v>0.2857003921721881</v>
       </c>
       <c r="S23" t="n">
-        <v>0.9869928059355442</v>
+        <v>0.1731432889018076</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Palantir Technologies Inc.</t>
+          <t>Gen Digital Inc.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>GEN</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>66.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="D24" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2183,26 +2183,28 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.3291712528765784</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
+        <v>0.1465900735417971</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-0.1008848813150681</v>
+      </c>
       <c r="H24" t="n">
-        <v>0.84796</v>
+        <v>0.7800700699999999</v>
       </c>
       <c r="I24" t="n">
-        <v>0.17292999</v>
+        <v>0.084910005</v>
       </c>
       <c r="J24" t="n">
-        <v>0.09952389147020013</v>
+        <v>0.09054857898215452</v>
       </c>
       <c r="K24" t="n">
-        <v>-0.3898353697011415</v>
+        <v>-0.4124256444150693</v>
       </c>
       <c r="L24" t="n">
-        <v>0.2552972336668627</v>
+        <v>0.2195512820512817</v>
       </c>
       <c r="M24" t="n">
-        <v>418925182976</v>
+        <v>18113243136</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -2215,39 +2217,39 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q24" t="b">
         <v>1</v>
       </c>
       <c r="R24" t="n">
-        <v>0.2862835047681325</v>
+        <v>0.2695654880786942</v>
       </c>
       <c r="S24" t="n">
-        <v>0.1092517037977452</v>
+        <v>0.4550608701426258</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DoorDash, Inc.</t>
+          <t>Palo Alto Networks, Inc.</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DASH</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>65.7</v>
+        <v>64.7</v>
       </c>
       <c r="D25" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -2255,30 +2257,32 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.2772574009717286</v>
-      </c>
-      <c r="G25" t="inlineStr"/>
+        <v>0.1853615538475797</v>
+      </c>
+      <c r="G25" t="n">
+        <v>-0.1450120266616515</v>
+      </c>
       <c r="H25" t="n">
-        <v>0.52225</v>
+        <v>0.70383</v>
       </c>
       <c r="I25" t="n">
-        <v>0.029719999</v>
+        <v>0.014040001</v>
       </c>
       <c r="J25" t="n">
-        <v>0.1988538704954423</v>
+        <v>0.1898381974897929</v>
       </c>
       <c r="K25" t="n">
-        <v>-0.3231946346762385</v>
+        <v>-0.5778920308483291</v>
       </c>
       <c r="L25" t="n">
-        <v>0.6152759023819964</v>
+        <v>0.32850115135022</v>
       </c>
       <c r="M25" t="n">
-        <v>91742175232</v>
+        <v>270471692288</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -2287,39 +2291,39 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q25" t="b">
         <v>1</v>
       </c>
       <c r="R25" t="n">
-        <v>0.350318824022277</v>
+        <v>0.1828783863643535</v>
       </c>
       <c r="S25" t="n">
-        <v>0.1817268398244434</v>
+        <v>0.9667499613356869</v>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Corpay, Inc.</t>
+          <t>Chipotle Mexican Grill, Inc.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CPAY</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>65.5</v>
+        <v>63.8</v>
       </c>
       <c r="D26" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2327,37 +2331,37 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.097332408585459</v>
+        <v>0.1136408299076579</v>
       </c>
       <c r="G26" t="n">
-        <v>0.06564477917470324</v>
+        <v>0.2116972328310951</v>
       </c>
       <c r="H26" t="n">
-        <v>0.8053900000000001</v>
+        <v>0.39361998</v>
       </c>
       <c r="I26" t="n">
-        <v>0.06315999999999999</v>
+        <v>0.13075</v>
       </c>
       <c r="J26" t="n">
-        <v>0.1071883180824746</v>
+        <v>0.2115850828729282</v>
       </c>
       <c r="K26" t="n">
-        <v>-0.392751639167087</v>
+        <v>-0.225414364640884</v>
       </c>
       <c r="L26" t="n">
-        <v>0.2729162844737966</v>
+        <v>0.9386495098039215</v>
       </c>
       <c r="M26" t="n">
-        <v>27338686464</v>
+        <v>45808132096</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Høj bruttomargin, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, positivt momentum</t>
         </is>
       </c>
       <c r="P26" t="n">
@@ -2367,33 +2371,33 @@
         <v>1</v>
       </c>
       <c r="R26" t="n">
-        <v>0.1983594200281382</v>
+        <v>0.1584000244140624</v>
       </c>
       <c r="S26" t="n">
-        <v>0.3243320712476749</v>
+        <v>0.1117935883330254</v>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dell Technologies Inc.</t>
+          <t>Super Micro Computer, Inc.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>63.7</v>
+        <v>63.1</v>
       </c>
       <c r="D27" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2401,28 +2405,28 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.03534983888485344</v>
+        <v>0.7634291720222148</v>
       </c>
       <c r="G27" t="n">
-        <v>0.388859258627138</v>
+        <v>0.4181552919037022</v>
       </c>
       <c r="H27" t="n">
-        <v>0.19893</v>
+        <v>0.108219996</v>
       </c>
       <c r="I27" t="n">
-        <v>0.08554</v>
+        <v>0.07877000000000001</v>
       </c>
       <c r="J27" t="n">
-        <v>0.07692276872591286</v>
+        <v>0.05673316708229414</v>
       </c>
       <c r="K27" t="n">
-        <v>-0.7897126721868203</v>
+        <v>-0.5142144638403989</v>
       </c>
       <c r="L27" t="n">
-        <v>0.09740602048705056</v>
+        <v>0.1103297769156157</v>
       </c>
       <c r="M27" t="n">
-        <v>338669076480</v>
+        <v>26344310784</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -2431,7 +2435,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Stærk eps-vækst, positivt momentum</t>
+          <t>Stærk omsætningsvækst, stærk eps-vækst, positivt momentum</t>
         </is>
       </c>
       <c r="P27" t="n">
@@ -2441,33 +2445,33 @@
         <v>1</v>
       </c>
       <c r="R27" t="n">
-        <v>0.3311851479129055</v>
+        <v>0.2543008863115785</v>
       </c>
       <c r="S27" t="n">
-        <v>2.595238758114921</v>
+        <v>0.2977345944714418</v>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Workday, Inc.</t>
+          <t>GoDaddy Inc.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>GDDY</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>63.7</v>
+        <v>63.1</v>
       </c>
       <c r="D28" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2475,71 +2479,73 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.1539697807235301</v>
-      </c>
-      <c r="G28" t="inlineStr"/>
+        <v>0.06564722266304868</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.4161701082120004</v>
+      </c>
       <c r="H28" t="n">
-        <v>0.75795</v>
+        <v>0.63802</v>
       </c>
       <c r="I28" t="n">
-        <v>0.04513</v>
+        <v>0.09882000000000001</v>
       </c>
       <c r="J28" t="n">
-        <v>0.05778073446039134</v>
+        <v>0.06590527174467242</v>
       </c>
       <c r="K28" t="n">
-        <v>-0.436334848562235</v>
+        <v>-0.2700112164780258</v>
       </c>
       <c r="L28" t="n">
-        <v>0.132422919349175</v>
+        <v>0.2440834592145025</v>
       </c>
       <c r="M28" t="n">
-        <v>47185387520</v>
+        <v>12420340736</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q28" t="b">
         <v>1</v>
       </c>
       <c r="R28" t="n">
-        <v>0.3570141041214594</v>
+        <v>0.3046428373512917</v>
       </c>
       <c r="S28" t="n">
-        <v>0.2962791445258133</v>
+        <v>0.2144891603074206</v>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lumentum Holdings Inc.</t>
+          <t>Global Payments Inc.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>GPN</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>63.6</v>
+        <v>62.9</v>
       </c>
       <c r="D29" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2547,71 +2553,73 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.1948193100306586</v>
-      </c>
-      <c r="G29" t="inlineStr"/>
+        <v>-0.0495682906305519</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1.435693379691408</v>
+      </c>
       <c r="H29" t="n">
-        <v>0.44244</v>
+        <v>0.63959</v>
       </c>
       <c r="I29" t="n">
-        <v>0.05815</v>
+        <v>0.023340002</v>
       </c>
       <c r="J29" t="n">
-        <v>0.3031795564280488</v>
+        <v>0.1712967493487372</v>
       </c>
       <c r="K29" t="n">
-        <v>-0.8360066042178484</v>
+        <v>-0.307282817986182</v>
       </c>
       <c r="L29" t="n">
-        <v>0.3626521069312577</v>
+        <v>0.5574563214154074</v>
       </c>
       <c r="M29" t="n">
-        <v>79048572928</v>
+        <v>23363158016</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Stærk omsætningsvækst, høj bruttomargin, positivt momentum</t>
+          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>88.88888888888889</v>
+        <v>100</v>
       </c>
       <c r="Q29" t="b">
         <v>1</v>
       </c>
       <c r="R29" t="n">
-        <v>0.02037263771090236</v>
+        <v>0.3581833609922469</v>
       </c>
       <c r="S29" t="n">
-        <v>0.5780656848186252</v>
+        <v>0.2633905888738934</v>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>News Corporation</t>
+          <t>Corpay, Inc.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>CPAY</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>61.9</v>
+        <v>62.8</v>
       </c>
       <c r="D30" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2619,37 +2627,37 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.0405993172034298</v>
+        <v>0.097332408585459</v>
       </c>
       <c r="G30" t="n">
-        <v>0.5822968332827563</v>
+        <v>0.06564477917470324</v>
       </c>
       <c r="H30" t="n">
-        <v>0.57167</v>
+        <v>0.8053900000000001</v>
       </c>
       <c r="I30" t="n">
-        <v>0.04658</v>
+        <v>0.06315999999999999</v>
       </c>
       <c r="J30" t="n">
-        <v>0.1899473511023364</v>
+        <v>0.1292930282690705</v>
       </c>
       <c r="K30" t="n">
-        <v>-0.2694965449160909</v>
+        <v>-0.3806280926951154</v>
       </c>
       <c r="L30" t="n">
-        <v>0.7048229548229551</v>
+        <v>0.3396833569313937</v>
       </c>
       <c r="M30" t="n">
-        <v>16310325248</v>
+        <v>26803562496</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Stærk eps-vækst, høj bruttomargin, positivt momentum</t>
+          <t>Høj bruttomargin, positivt momentum</t>
         </is>
       </c>
       <c r="P30" t="n">
@@ -2659,33 +2667,33 @@
         <v>1</v>
       </c>
       <c r="R30" t="n">
-        <v>0.1148202176994255</v>
+        <v>0.1635171558191761</v>
       </c>
       <c r="S30" t="n">
-        <v>0.239520454510977</v>
+        <v>0.269498707302106</v>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Gen Digital Inc.</t>
+          <t>Lumentum Holdings Inc.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GEN</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>60.9</v>
+        <v>62.8</v>
       </c>
       <c r="D31" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2693,28 +2701,26 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.1465900735417971</v>
-      </c>
-      <c r="G31" t="n">
-        <v>-0.1008848813150681</v>
-      </c>
+        <v>0.1948193100306586</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>0.7800700699999999</v>
+        <v>0.44244</v>
       </c>
       <c r="I31" t="n">
-        <v>0.084910005</v>
+        <v>0.05815</v>
       </c>
       <c r="J31" t="n">
-        <v>0.07667210440456773</v>
+        <v>0.2398508138895181</v>
       </c>
       <c r="K31" t="n">
-        <v>-0.4199021207177813</v>
+        <v>-0.8441042900445509</v>
       </c>
       <c r="L31" t="n">
-        <v>0.1825951825951827</v>
+        <v>0.2841483175933854</v>
       </c>
       <c r="M31" t="n">
-        <v>18346690560</v>
+        <v>83154591744</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -2727,20 +2733,20 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="Q31" t="b">
         <v>1</v>
       </c>
       <c r="R31" t="n">
-        <v>0.1714275925138224</v>
+        <v>0.04208680550719479</v>
       </c>
       <c r="S31" t="n">
-        <v>0.3688674871134887</v>
+        <v>0.5046989707469345</v>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>2026-09-06 11:35:57</t>
+          <t>2026-09-13 12:39:07</t>
         </is>
       </c>
     </row>

</xml_diff>